<commit_message>
add matrix for 2nd session + redid the graph
</commit_message>
<xml_diff>
--- a/interaction_matrix.xlsx
+++ b/interaction_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\stage_Curtin_Mahidol_2026\bobtail_pilot\bobtail_interactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{875AAAD6-28A2-41D3-880A-C90877A29E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACE3679-6ACA-4292-A87A-7D4AB2A77136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1281983F-7B2F-482E-A56E-54D10BC5CD37}"/>
   </bookViews>
@@ -169,7 +169,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -347,6 +347,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -510,8 +516,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -891,7 +898,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1">
+      <c r="A1" s="1">
         <v>0</v>
       </c>
       <c r="B1">
@@ -923,7 +930,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>0</v>
       </c>
       <c r="C2">
@@ -955,7 +962,7 @@
       <c r="B3">
         <v>2</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>0</v>
       </c>
       <c r="D3">
@@ -987,7 +994,7 @@
       <c r="C4">
         <v>2</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>0</v>
       </c>
       <c r="E4">
@@ -1017,9 +1024,9 @@
         <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1">
         <v>0</v>
       </c>
       <c r="F5">
@@ -1051,7 +1058,7 @@
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="1">
         <v>0</v>
       </c>
       <c r="G6">
@@ -1083,7 +1090,7 @@
       <c r="F7">
         <v>0</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="1">
         <v>0</v>
       </c>
       <c r="H7">
@@ -1115,7 +1122,7 @@
       <c r="G8">
         <v>0</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="1">
         <v>0</v>
       </c>
       <c r="I8">
@@ -1147,7 +1154,7 @@
       <c r="H9">
         <v>0</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>